<commit_message>
🔄 Auto-collect traffic data: 2026-09-13 10:24 AM IST
</commit_message>
<xml_diff>
--- a/output/excel/Bus_vs_Metro_Data_2026-09-13_Sun.xlsx
+++ b/output/excel/Bus_vs_Metro_Data_2026-09-13_Sun.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="All Periods Combined" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2222" uniqueCount="506">
   <si>
     <t>Date</t>
   </si>
@@ -140,7 +141,7 @@
     <t>12:00 AM</t>
   </si>
   <si>
-    <t>Saturday (Weekend) - Night Off-Peak</t>
+    <t>Sunday (Weekend) - Night Off-Peak</t>
   </si>
   <si>
     <t>34B</t>
@@ -983,6 +984,471 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/12_00_AM/MC-25/car.jpg</t>
   </si>
   <si>
+    <t>9/13/2026, 10:02:25 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>Sunday (Weekend) - Morning Peak</t>
+  </si>
+  <si>
+    <t> | 50 min | 10:00 AM—10:50 AM | DN-9/1  234/1 | 10:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:00 AM—10:28 AM | Blue Line | 10:00 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>22 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.79x</t>
+  </si>
+  <si>
+    <t>44.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-01/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:02:54 AM</t>
+  </si>
+  <si>
+    <t> | 51 min | 10:04 AM—10:55 AM | S-112 | 10:04 AM from Khudiram Metro | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:08 AM—10:36 AM | Blue Line | 10:08 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-02/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:03:21 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:07 AM—10:19 AM | S-168 | 10:07 AM from Dumdum Station | Details</t>
+  </si>
+  <si>
+    <t> | 7 min | 10:07 AM—10:14 AM | Blue Line | 10:07 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1.71x</t>
+  </si>
+  <si>
+    <t>41.7% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-03/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:03:49 AM</t>
+  </si>
+  <si>
+    <t>S-10</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:05 AM—10:23 AM | S-10 | 10:05 AM from Shyambazar | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:06 AM—10:17 AM | Blue Line | 10:06 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-04/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:04:17 AM</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:04 AM—10:22 AM | 40A | 10:04 AM from S.P. Mukherjee Road / R.B. Avenue Crossing | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:13 AM—10:24 AM | Blue Line | 10:13 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-05/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:04:43 AM</t>
+  </si>
+  <si>
+    <t> | 24 min | 10:00 AM—10:24 AM | DN-9/1 | 10:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:00 AM—10:12 AM | Blue Line | 10:00 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-06/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:05:11 AM</t>
+  </si>
+  <si>
+    <t> | 27 min | 10:11 AM—10:38 AM | 12C/1B | 10:11 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 10:05 AM—10:22 AM | Blue Line | 10:05 AM from Esplanade | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>1.59x</t>
+  </si>
+  <si>
+    <t>37.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-07/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:05:40 AM</t>
+  </si>
+  <si>
+    <t> | 22 min | 10:09 AM—10:31 AM | S-112 | 10:09 AM from Tollygunge Tram Depot | Details</t>
+  </si>
+  <si>
+    <t> | 14 min | 10:10 AM—10:24 AM | Blue Line | 10:10 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-08/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:06:07 AM</t>
+  </si>
+  <si>
+    <t> | 36 min | 10:00 AM—10:36 AM | 30B   | 10:00 AM from Dumdum Station |  3 min | Details</t>
+  </si>
+  <si>
+    <t> | 16 min | 10:01 AM—10:17 AM | Blue Line | 10:01 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-09/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:06:35 AM</t>
+  </si>
+  <si>
+    <t> | 40 min | 10:00 AM—10:40 AM | 215A/1 | 10:00 AM from Howrah Station | Details</t>
+  </si>
+  <si>
+    <t> | 30 min | 10:02 AM—10:32 AM | Green Line | 10:02 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>25.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-10/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:07:03 AM</t>
+  </si>
+  <si>
+    <t>S-12</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:02 AM—10:28 AM | S-12 | 10:02 AM from Sealdah - B.R. Singh Hospital | Details</t>
+  </si>
+  <si>
+    <t> | 22 min | 10:10 AM—10:32 AM | Green Line | 10:10 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>Tie</t>
+  </si>
+  <si>
+    <t>0%</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-11/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:07:30 AM</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>Walk &gt; Bus Walk</t>
+  </si>
+  <si>
+    <t> | 27 min | 10:00 AM—10:27 AM |   72 </t>
+  </si>
+  <si>
+    <t> | 10 min | 10:00 AM—10:10 AM | Green Line | 10:00 AM from Howrah Maidan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>2.70x</t>
+  </si>
+  <si>
+    <t>63.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-12/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:07:58 AM</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:02 AM—10:28 AM | S-21  S-12 | 10:02 AM from Phoolbagan | Details</t>
+  </si>
+  <si>
+    <t> | 19 min | 10:13 AM—10:32 AM | Green Line | 10:13 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-13/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:08:27 AM</t>
+  </si>
+  <si>
+    <t> | 29 min | 10:00 AM—10:29 AM | 44/1 | 10:00 AM from Howrah Station |  2 min | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:02 AM—10:13 AM | Green Line | 10:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-14/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:08:55 AM</t>
+  </si>
+  <si>
+    <t> | 34 min | 10:20 AM—10:54 AM | S-12N | 10:20 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 25 min | 10:07 AM—10:32 AM | Green Line | 10:07 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-15/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:10:37 AM</t>
+  </si>
+  <si>
+    <t>AS-3</t>
+  </si>
+  <si>
+    <t> | 36 min | 10:03 AM—10:39 AM | AS-3 | 10:03 AM from Dhalai Bridge | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-16/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:12:15 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 10:00 AM—10:16 AM | V-1 | 10:00 AM from Ruby | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-17/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:13:55 AM</t>
+  </si>
+  <si>
+    <t>C26A</t>
+  </si>
+  <si>
+    <t> | 47 min | 10:02 AM—10:49 AM |   C26A</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-18/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:15:34 AM</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:01 AM—10:27 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-19/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:17:14 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:01 AM—10:13 AM | 222 | 10:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-20/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:18:56 AM</t>
+  </si>
+  <si>
+    <t> | 14 min | 10:01 AM—10:15 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-21/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:20:37 AM</t>
+  </si>
+  <si>
+    <t> | 22 min | 10:01 AM—10:23 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-22/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:22:17 AM</t>
+  </si>
+  <si>
+    <t> | 8 min | 10:01 AM—10:09 AM | 222 | 10:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-23/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:23:59 AM</t>
+  </si>
+  <si>
+    <t> | 4 min | 10:01 AM—10:05 AM | S-3B | 10:01 AM from Pathak Para | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-24/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-24/car.jpg</t>
+  </si>
+  <si>
+    <t>9/13/2026, 10:24:26 AM</t>
+  </si>
+  <si>
+    <t>DN-18</t>
+  </si>
+  <si>
+    <t> | 25 min | 10:05 AM—10:30 AM |   DN-18</t>
+  </si>
+  <si>
+    <t> | 7 min | 10:03 AM—10:10 AM | Yellow Line | 10:03 AM from Dum Dum Cantonment | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>3.57x</t>
+  </si>
+  <si>
+    <t>72.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-25/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-25/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-13/10_00_AM/MC-25/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1023,6 +1489,48 @@
   </si>
   <si>
     <t>12:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>10:00 AM Scraped At</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Bus</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Metro</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Car (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Faster Mode</t>
+  </si>
+  <si>
+    <t>10:00 AM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -4078,10 +4586,2638 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:AF26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>324</v>
+      </c>
+      <c r="K2" t="s">
+        <v>325</v>
+      </c>
+      <c r="L2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2">
+        <v>50</v>
+      </c>
+      <c r="O2" t="s">
+        <v>192</v>
+      </c>
+      <c r="P2" t="s">
+        <v>326</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" t="s">
+        <v>327</v>
+      </c>
+      <c r="V2">
+        <v>33</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="X2" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>330</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>331</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>332</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>324</v>
+      </c>
+      <c r="K3" t="s">
+        <v>325</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3">
+        <v>51</v>
+      </c>
+      <c r="O3" t="s">
+        <v>62</v>
+      </c>
+      <c r="P3" t="s">
+        <v>335</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S3">
+        <v>28</v>
+      </c>
+      <c r="T3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U3" t="s">
+        <v>336</v>
+      </c>
+      <c r="V3">
+        <v>31</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="X3" t="s">
+        <v>66</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>337</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>338</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>340</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I4" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" t="s">
+        <v>324</v>
+      </c>
+      <c r="K4" t="s">
+        <v>325</v>
+      </c>
+      <c r="L4" t="s">
+        <v>76</v>
+      </c>
+      <c r="M4" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4">
+        <v>12</v>
+      </c>
+      <c r="O4" t="s">
+        <v>62</v>
+      </c>
+      <c r="P4" t="s">
+        <v>341</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R4" t="s">
+        <v>44</v>
+      </c>
+      <c r="S4">
+        <v>7</v>
+      </c>
+      <c r="T4" t="s">
+        <v>48</v>
+      </c>
+      <c r="U4" t="s">
+        <v>342</v>
+      </c>
+      <c r="V4">
+        <v>15</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="X4" t="s">
+        <v>343</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>344</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>345</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>346</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>348</v>
+      </c>
+      <c r="D5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>324</v>
+      </c>
+      <c r="K5" t="s">
+        <v>325</v>
+      </c>
+      <c r="L5" t="s">
+        <v>349</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5">
+        <v>18</v>
+      </c>
+      <c r="O5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P5" t="s">
+        <v>350</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R5" t="s">
+        <v>44</v>
+      </c>
+      <c r="S5">
+        <v>11</v>
+      </c>
+      <c r="T5" t="s">
+        <v>48</v>
+      </c>
+      <c r="U5" t="s">
+        <v>351</v>
+      </c>
+      <c r="V5">
+        <v>15</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="X5" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>352</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>353</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>355</v>
+      </c>
+      <c r="D6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" t="s">
+        <v>99</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>324</v>
+      </c>
+      <c r="K6" t="s">
+        <v>325</v>
+      </c>
+      <c r="L6" t="s">
+        <v>100</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N6">
+        <v>18</v>
+      </c>
+      <c r="O6" t="s">
+        <v>62</v>
+      </c>
+      <c r="P6" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>47</v>
+      </c>
+      <c r="R6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S6">
+        <v>11</v>
+      </c>
+      <c r="T6" t="s">
+        <v>48</v>
+      </c>
+      <c r="U6" t="s">
+        <v>357</v>
+      </c>
+      <c r="V6">
+        <v>14</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="X6" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>358</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>359</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>361</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" t="s">
+        <v>324</v>
+      </c>
+      <c r="K7" t="s">
+        <v>325</v>
+      </c>
+      <c r="L7" t="s">
+        <v>62</v>
+      </c>
+      <c r="M7" t="s">
+        <v>44</v>
+      </c>
+      <c r="N7">
+        <v>24</v>
+      </c>
+      <c r="O7" t="s">
+        <v>62</v>
+      </c>
+      <c r="P7" t="s">
+        <v>362</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S7">
+        <v>12</v>
+      </c>
+      <c r="T7" t="s">
+        <v>48</v>
+      </c>
+      <c r="U7" t="s">
+        <v>363</v>
+      </c>
+      <c r="V7">
+        <v>23</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="X7" t="s">
+        <v>111</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>364</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>365</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>367</v>
+      </c>
+      <c r="D8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" t="s">
+        <v>118</v>
+      </c>
+      <c r="J8" t="s">
+        <v>324</v>
+      </c>
+      <c r="K8" t="s">
+        <v>325</v>
+      </c>
+      <c r="L8" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" t="s">
+        <v>44</v>
+      </c>
+      <c r="N8">
+        <v>27</v>
+      </c>
+      <c r="O8" t="s">
+        <v>62</v>
+      </c>
+      <c r="P8" t="s">
+        <v>368</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R8" t="s">
+        <v>44</v>
+      </c>
+      <c r="S8">
+        <v>17</v>
+      </c>
+      <c r="T8" t="s">
+        <v>48</v>
+      </c>
+      <c r="U8" t="s">
+        <v>369</v>
+      </c>
+      <c r="V8">
+        <v>23</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X8" t="s">
+        <v>370</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>371</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>372</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>373</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>375</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9" t="s">
+        <v>118</v>
+      </c>
+      <c r="I9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
+        <v>324</v>
+      </c>
+      <c r="K9" t="s">
+        <v>325</v>
+      </c>
+      <c r="L9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" t="s">
+        <v>44</v>
+      </c>
+      <c r="N9">
+        <v>22</v>
+      </c>
+      <c r="O9" t="s">
+        <v>62</v>
+      </c>
+      <c r="P9" t="s">
+        <v>376</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>47</v>
+      </c>
+      <c r="R9" t="s">
+        <v>44</v>
+      </c>
+      <c r="S9">
+        <v>14</v>
+      </c>
+      <c r="T9" t="s">
+        <v>48</v>
+      </c>
+      <c r="U9" t="s">
+        <v>377</v>
+      </c>
+      <c r="V9">
+        <v>22</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="X9" t="s">
+        <v>286</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>287</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>378</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>379</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>381</v>
+      </c>
+      <c r="D10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" t="s">
+        <v>74</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" t="s">
+        <v>324</v>
+      </c>
+      <c r="K10" t="s">
+        <v>325</v>
+      </c>
+      <c r="L10" t="s">
+        <v>140</v>
+      </c>
+      <c r="M10" t="s">
+        <v>44</v>
+      </c>
+      <c r="N10">
+        <v>36</v>
+      </c>
+      <c r="O10" t="s">
+        <v>141</v>
+      </c>
+      <c r="P10" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>47</v>
+      </c>
+      <c r="R10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>48</v>
+      </c>
+      <c r="U10" t="s">
+        <v>383</v>
+      </c>
+      <c r="V10">
+        <v>29</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="X10" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>384</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>385</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>387</v>
+      </c>
+      <c r="D11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>154</v>
+      </c>
+      <c r="I11" t="s">
+        <v>155</v>
+      </c>
+      <c r="J11" t="s">
+        <v>324</v>
+      </c>
+      <c r="K11" t="s">
+        <v>325</v>
+      </c>
+      <c r="L11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M11" t="s">
+        <v>44</v>
+      </c>
+      <c r="N11">
+        <v>40</v>
+      </c>
+      <c r="O11" t="s">
+        <v>62</v>
+      </c>
+      <c r="P11" t="s">
+        <v>388</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>157</v>
+      </c>
+      <c r="R11" t="s">
+        <v>44</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>48</v>
+      </c>
+      <c r="U11" t="s">
+        <v>389</v>
+      </c>
+      <c r="V11">
+        <v>39</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X11" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>390</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>391</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>392</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>394</v>
+      </c>
+      <c r="D12" t="s">
+        <v>166</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" t="s">
+        <v>153</v>
+      </c>
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" t="s">
+        <v>167</v>
+      </c>
+      <c r="I12" t="s">
+        <v>155</v>
+      </c>
+      <c r="J12" t="s">
+        <v>324</v>
+      </c>
+      <c r="K12" t="s">
+        <v>325</v>
+      </c>
+      <c r="L12" t="s">
+        <v>395</v>
+      </c>
+      <c r="M12" t="s">
+        <v>44</v>
+      </c>
+      <c r="N12">
+        <v>26</v>
+      </c>
+      <c r="O12" t="s">
+        <v>62</v>
+      </c>
+      <c r="P12" t="s">
+        <v>396</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>157</v>
+      </c>
+      <c r="R12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S12">
+        <v>22</v>
+      </c>
+      <c r="T12" t="s">
+        <v>48</v>
+      </c>
+      <c r="U12" t="s">
+        <v>397</v>
+      </c>
+      <c r="V12">
+        <v>22</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="X12" t="s">
+        <v>172</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>398</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>399</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>400</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>401</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
+        <v>403</v>
+      </c>
+      <c r="D13" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" t="s">
+        <v>154</v>
+      </c>
+      <c r="I13" t="s">
+        <v>167</v>
+      </c>
+      <c r="J13" t="s">
+        <v>324</v>
+      </c>
+      <c r="K13" t="s">
+        <v>325</v>
+      </c>
+      <c r="L13" t="s">
+        <v>404</v>
+      </c>
+      <c r="M13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N13">
+        <v>27</v>
+      </c>
+      <c r="O13" t="s">
+        <v>405</v>
+      </c>
+      <c r="P13" t="s">
+        <v>406</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>157</v>
+      </c>
+      <c r="R13" t="s">
+        <v>44</v>
+      </c>
+      <c r="S13">
+        <v>10</v>
+      </c>
+      <c r="T13" t="s">
+        <v>48</v>
+      </c>
+      <c r="U13" t="s">
+        <v>407</v>
+      </c>
+      <c r="V13">
+        <v>21</v>
+      </c>
+      <c r="W13" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="X13" t="s">
+        <v>408</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>409</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>410</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>411</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>413</v>
+      </c>
+      <c r="D14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" t="s">
+        <v>179</v>
+      </c>
+      <c r="G14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J14" t="s">
+        <v>324</v>
+      </c>
+      <c r="K14" t="s">
+        <v>325</v>
+      </c>
+      <c r="L14" t="s">
+        <v>191</v>
+      </c>
+      <c r="M14" t="s">
+        <v>44</v>
+      </c>
+      <c r="N14">
+        <v>26</v>
+      </c>
+      <c r="O14" t="s">
+        <v>192</v>
+      </c>
+      <c r="P14" t="s">
+        <v>414</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>157</v>
+      </c>
+      <c r="R14" t="s">
+        <v>44</v>
+      </c>
+      <c r="S14">
+        <v>19</v>
+      </c>
+      <c r="T14" t="s">
+        <v>48</v>
+      </c>
+      <c r="U14" t="s">
+        <v>415</v>
+      </c>
+      <c r="V14">
+        <v>17</v>
+      </c>
+      <c r="W14" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="X14" t="s">
+        <v>255</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>256</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>416</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>417</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>419</v>
+      </c>
+      <c r="D15" t="s">
+        <v>202</v>
+      </c>
+      <c r="E15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" t="s">
+        <v>154</v>
+      </c>
+      <c r="I15" t="s">
+        <v>190</v>
+      </c>
+      <c r="J15" t="s">
+        <v>324</v>
+      </c>
+      <c r="K15" t="s">
+        <v>325</v>
+      </c>
+      <c r="L15" t="s">
+        <v>62</v>
+      </c>
+      <c r="M15" t="s">
+        <v>44</v>
+      </c>
+      <c r="N15">
+        <v>29</v>
+      </c>
+      <c r="O15" t="s">
+        <v>62</v>
+      </c>
+      <c r="P15" t="s">
+        <v>420</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>157</v>
+      </c>
+      <c r="R15" t="s">
+        <v>44</v>
+      </c>
+      <c r="S15">
+        <v>11</v>
+      </c>
+      <c r="T15" t="s">
+        <v>48</v>
+      </c>
+      <c r="U15" t="s">
+        <v>421</v>
+      </c>
+      <c r="V15">
+        <v>25</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="X15" t="s">
+        <v>206</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>207</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>422</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>423</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>425</v>
+      </c>
+      <c r="D16" t="s">
+        <v>212</v>
+      </c>
+      <c r="E16" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J16" t="s">
+        <v>324</v>
+      </c>
+      <c r="K16" t="s">
+        <v>325</v>
+      </c>
+      <c r="L16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M16" t="s">
+        <v>44</v>
+      </c>
+      <c r="N16">
+        <v>34</v>
+      </c>
+      <c r="O16" t="s">
+        <v>62</v>
+      </c>
+      <c r="P16" t="s">
+        <v>426</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>157</v>
+      </c>
+      <c r="R16" t="s">
+        <v>44</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>48</v>
+      </c>
+      <c r="U16" t="s">
+        <v>427</v>
+      </c>
+      <c r="V16">
+        <v>24</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="X16" t="s">
+        <v>216</v>
+      </c>
+      <c r="Y16" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>217</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>428</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>429</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>431</v>
+      </c>
+      <c r="D17" t="s">
+        <v>222</v>
+      </c>
+      <c r="E17" t="s">
+        <v>223</v>
+      </c>
+      <c r="F17" t="s">
+        <v>224</v>
+      </c>
+      <c r="G17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" t="s">
+        <v>130</v>
+      </c>
+      <c r="I17" t="s">
+        <v>225</v>
+      </c>
+      <c r="J17" t="s">
+        <v>324</v>
+      </c>
+      <c r="K17" t="s">
+        <v>325</v>
+      </c>
+      <c r="L17" t="s">
+        <v>432</v>
+      </c>
+      <c r="M17" t="s">
+        <v>44</v>
+      </c>
+      <c r="N17">
+        <v>36</v>
+      </c>
+      <c r="O17" t="s">
+        <v>62</v>
+      </c>
+      <c r="P17" t="s">
+        <v>433</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>44</v>
+      </c>
+      <c r="R17" t="s">
+        <v>44</v>
+      </c>
+      <c r="S17" t="s">
+        <v>228</v>
+      </c>
+      <c r="T17" t="s">
+        <v>44</v>
+      </c>
+      <c r="U17" t="s">
+        <v>44</v>
+      </c>
+      <c r="V17">
+        <v>20</v>
+      </c>
+      <c r="W17" t="s">
+        <v>44</v>
+      </c>
+      <c r="X17" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>434</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>436</v>
+      </c>
+      <c r="D18" t="s">
+        <v>232</v>
+      </c>
+      <c r="E18" t="s">
+        <v>223</v>
+      </c>
+      <c r="F18" t="s">
+        <v>179</v>
+      </c>
+      <c r="G18" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" t="s">
+        <v>233</v>
+      </c>
+      <c r="I18" t="s">
+        <v>225</v>
+      </c>
+      <c r="J18" t="s">
+        <v>324</v>
+      </c>
+      <c r="K18" t="s">
+        <v>325</v>
+      </c>
+      <c r="L18" t="s">
+        <v>234</v>
+      </c>
+      <c r="M18" t="s">
+        <v>44</v>
+      </c>
+      <c r="N18">
+        <v>16</v>
+      </c>
+      <c r="O18" t="s">
+        <v>62</v>
+      </c>
+      <c r="P18" t="s">
+        <v>437</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>44</v>
+      </c>
+      <c r="R18" t="s">
+        <v>44</v>
+      </c>
+      <c r="S18" t="s">
+        <v>228</v>
+      </c>
+      <c r="T18" t="s">
+        <v>44</v>
+      </c>
+      <c r="U18" t="s">
+        <v>44</v>
+      </c>
+      <c r="V18">
+        <v>8</v>
+      </c>
+      <c r="W18" t="s">
+        <v>44</v>
+      </c>
+      <c r="X18" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>438</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D19" t="s">
+        <v>239</v>
+      </c>
+      <c r="E19" t="s">
+        <v>223</v>
+      </c>
+      <c r="F19" t="s">
+        <v>224</v>
+      </c>
+      <c r="G19" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" t="s">
+        <v>240</v>
+      </c>
+      <c r="J19" t="s">
+        <v>324</v>
+      </c>
+      <c r="K19" t="s">
+        <v>325</v>
+      </c>
+      <c r="L19" t="s">
+        <v>441</v>
+      </c>
+      <c r="M19" t="s">
+        <v>44</v>
+      </c>
+      <c r="N19">
+        <v>47</v>
+      </c>
+      <c r="O19" t="s">
+        <v>45</v>
+      </c>
+      <c r="P19" t="s">
+        <v>442</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>44</v>
+      </c>
+      <c r="R19" t="s">
+        <v>44</v>
+      </c>
+      <c r="S19" t="s">
+        <v>228</v>
+      </c>
+      <c r="T19" t="s">
+        <v>44</v>
+      </c>
+      <c r="U19" t="s">
+        <v>44</v>
+      </c>
+      <c r="V19">
+        <v>18</v>
+      </c>
+      <c r="W19" t="s">
+        <v>44</v>
+      </c>
+      <c r="X19" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>443</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D20" t="s">
+        <v>246</v>
+      </c>
+      <c r="E20" t="s">
+        <v>247</v>
+      </c>
+      <c r="F20" t="s">
+        <v>248</v>
+      </c>
+      <c r="G20" t="s">
+        <v>38</v>
+      </c>
+      <c r="H20" t="s">
+        <v>249</v>
+      </c>
+      <c r="I20" t="s">
+        <v>250</v>
+      </c>
+      <c r="J20" t="s">
+        <v>324</v>
+      </c>
+      <c r="K20" t="s">
+        <v>325</v>
+      </c>
+      <c r="L20" t="s">
+        <v>251</v>
+      </c>
+      <c r="M20" t="s">
+        <v>44</v>
+      </c>
+      <c r="N20">
+        <v>26</v>
+      </c>
+      <c r="O20" t="s">
+        <v>62</v>
+      </c>
+      <c r="P20" t="s">
+        <v>446</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>44</v>
+      </c>
+      <c r="R20" t="s">
+        <v>44</v>
+      </c>
+      <c r="S20" t="s">
+        <v>228</v>
+      </c>
+      <c r="T20" t="s">
+        <v>44</v>
+      </c>
+      <c r="U20" t="s">
+        <v>44</v>
+      </c>
+      <c r="V20">
+        <v>21</v>
+      </c>
+      <c r="W20" t="s">
+        <v>44</v>
+      </c>
+      <c r="X20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>447</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
+        <v>449</v>
+      </c>
+      <c r="D21" t="s">
+        <v>261</v>
+      </c>
+      <c r="E21" t="s">
+        <v>247</v>
+      </c>
+      <c r="F21" t="s">
+        <v>179</v>
+      </c>
+      <c r="G21" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21" t="s">
+        <v>262</v>
+      </c>
+      <c r="I21" t="s">
+        <v>250</v>
+      </c>
+      <c r="J21" t="s">
+        <v>324</v>
+      </c>
+      <c r="K21" t="s">
+        <v>325</v>
+      </c>
+      <c r="L21" t="s">
+        <v>293</v>
+      </c>
+      <c r="M21" t="s">
+        <v>44</v>
+      </c>
+      <c r="N21">
+        <v>12</v>
+      </c>
+      <c r="O21" t="s">
+        <v>62</v>
+      </c>
+      <c r="P21" t="s">
+        <v>450</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>44</v>
+      </c>
+      <c r="R21" t="s">
+        <v>44</v>
+      </c>
+      <c r="S21" t="s">
+        <v>228</v>
+      </c>
+      <c r="T21" t="s">
+        <v>44</v>
+      </c>
+      <c r="U21" t="s">
+        <v>44</v>
+      </c>
+      <c r="V21">
+        <v>10</v>
+      </c>
+      <c r="W21" t="s">
+        <v>44</v>
+      </c>
+      <c r="X21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>451</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s">
+        <v>453</v>
+      </c>
+      <c r="D22" t="s">
+        <v>271</v>
+      </c>
+      <c r="E22" t="s">
+        <v>247</v>
+      </c>
+      <c r="F22" t="s">
+        <v>179</v>
+      </c>
+      <c r="G22" t="s">
+        <v>73</v>
+      </c>
+      <c r="H22" t="s">
+        <v>249</v>
+      </c>
+      <c r="I22" t="s">
+        <v>262</v>
+      </c>
+      <c r="J22" t="s">
+        <v>324</v>
+      </c>
+      <c r="K22" t="s">
+        <v>325</v>
+      </c>
+      <c r="L22" t="s">
+        <v>251</v>
+      </c>
+      <c r="M22" t="s">
+        <v>44</v>
+      </c>
+      <c r="N22">
+        <v>14</v>
+      </c>
+      <c r="O22" t="s">
+        <v>62</v>
+      </c>
+      <c r="P22" t="s">
+        <v>454</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>44</v>
+      </c>
+      <c r="R22" t="s">
+        <v>44</v>
+      </c>
+      <c r="S22" t="s">
+        <v>228</v>
+      </c>
+      <c r="T22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U22" t="s">
+        <v>44</v>
+      </c>
+      <c r="V22">
+        <v>11</v>
+      </c>
+      <c r="W22" t="s">
+        <v>44</v>
+      </c>
+      <c r="X22" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>455</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>457</v>
+      </c>
+      <c r="D23" t="s">
+        <v>281</v>
+      </c>
+      <c r="E23" t="s">
+        <v>247</v>
+      </c>
+      <c r="F23" t="s">
+        <v>248</v>
+      </c>
+      <c r="G23" t="s">
+        <v>73</v>
+      </c>
+      <c r="H23" t="s">
+        <v>249</v>
+      </c>
+      <c r="I23" t="s">
+        <v>282</v>
+      </c>
+      <c r="J23" t="s">
+        <v>324</v>
+      </c>
+      <c r="K23" t="s">
+        <v>325</v>
+      </c>
+      <c r="L23" t="s">
+        <v>251</v>
+      </c>
+      <c r="M23" t="s">
+        <v>44</v>
+      </c>
+      <c r="N23">
+        <v>22</v>
+      </c>
+      <c r="O23" t="s">
+        <v>62</v>
+      </c>
+      <c r="P23" t="s">
+        <v>458</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>44</v>
+      </c>
+      <c r="R23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S23" t="s">
+        <v>228</v>
+      </c>
+      <c r="T23" t="s">
+        <v>44</v>
+      </c>
+      <c r="U23" t="s">
+        <v>44</v>
+      </c>
+      <c r="V23">
+        <v>18</v>
+      </c>
+      <c r="W23" t="s">
+        <v>44</v>
+      </c>
+      <c r="X23" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>459</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>461</v>
+      </c>
+      <c r="D24" t="s">
+        <v>292</v>
+      </c>
+      <c r="E24" t="s">
+        <v>247</v>
+      </c>
+      <c r="F24" t="s">
+        <v>248</v>
+      </c>
+      <c r="G24" t="s">
+        <v>73</v>
+      </c>
+      <c r="H24" t="s">
+        <v>262</v>
+      </c>
+      <c r="I24" t="s">
+        <v>282</v>
+      </c>
+      <c r="J24" t="s">
+        <v>324</v>
+      </c>
+      <c r="K24" t="s">
+        <v>325</v>
+      </c>
+      <c r="L24" t="s">
+        <v>293</v>
+      </c>
+      <c r="M24" t="s">
+        <v>44</v>
+      </c>
+      <c r="N24">
+        <v>8</v>
+      </c>
+      <c r="O24" t="s">
+        <v>62</v>
+      </c>
+      <c r="P24" t="s">
+        <v>462</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>44</v>
+      </c>
+      <c r="R24" t="s">
+        <v>44</v>
+      </c>
+      <c r="S24" t="s">
+        <v>228</v>
+      </c>
+      <c r="T24" t="s">
+        <v>44</v>
+      </c>
+      <c r="U24" t="s">
+        <v>44</v>
+      </c>
+      <c r="V24">
+        <v>7</v>
+      </c>
+      <c r="W24" t="s">
+        <v>44</v>
+      </c>
+      <c r="X24" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>463</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>465</v>
+      </c>
+      <c r="D25" t="s">
+        <v>298</v>
+      </c>
+      <c r="E25" t="s">
+        <v>247</v>
+      </c>
+      <c r="F25" t="s">
+        <v>248</v>
+      </c>
+      <c r="G25" t="s">
+        <v>73</v>
+      </c>
+      <c r="H25" t="s">
+        <v>282</v>
+      </c>
+      <c r="I25" t="s">
+        <v>250</v>
+      </c>
+      <c r="J25" t="s">
+        <v>324</v>
+      </c>
+      <c r="K25" t="s">
+        <v>325</v>
+      </c>
+      <c r="L25" t="s">
+        <v>62</v>
+      </c>
+      <c r="M25" t="s">
+        <v>44</v>
+      </c>
+      <c r="N25">
+        <v>4</v>
+      </c>
+      <c r="O25" t="s">
+        <v>62</v>
+      </c>
+      <c r="P25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>44</v>
+      </c>
+      <c r="R25" t="s">
+        <v>44</v>
+      </c>
+      <c r="S25" t="s">
+        <v>228</v>
+      </c>
+      <c r="T25" t="s">
+        <v>44</v>
+      </c>
+      <c r="U25" t="s">
+        <v>44</v>
+      </c>
+      <c r="V25">
+        <v>3</v>
+      </c>
+      <c r="W25" t="s">
+        <v>44</v>
+      </c>
+      <c r="X25" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>467</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>228</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>469</v>
+      </c>
+      <c r="D26" t="s">
+        <v>308</v>
+      </c>
+      <c r="E26" t="s">
+        <v>309</v>
+      </c>
+      <c r="F26" t="s">
+        <v>310</v>
+      </c>
+      <c r="G26" t="s">
+        <v>73</v>
+      </c>
+      <c r="H26" t="s">
+        <v>311</v>
+      </c>
+      <c r="I26" t="s">
+        <v>312</v>
+      </c>
+      <c r="J26" t="s">
+        <v>324</v>
+      </c>
+      <c r="K26" t="s">
+        <v>325</v>
+      </c>
+      <c r="L26" t="s">
+        <v>470</v>
+      </c>
+      <c r="M26" t="s">
+        <v>44</v>
+      </c>
+      <c r="N26">
+        <v>25</v>
+      </c>
+      <c r="O26" t="s">
+        <v>45</v>
+      </c>
+      <c r="P26" t="s">
+        <v>471</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>315</v>
+      </c>
+      <c r="R26" t="s">
+        <v>44</v>
+      </c>
+      <c r="S26">
+        <v>7</v>
+      </c>
+      <c r="T26" t="s">
+        <v>48</v>
+      </c>
+      <c r="U26" t="s">
+        <v>472</v>
+      </c>
+      <c r="V26">
+        <v>13</v>
+      </c>
+      <c r="W26" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="X26" t="s">
+        <v>473</v>
+      </c>
+      <c r="Y26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>474</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>475</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>476</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>477</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AF1"/>
+  <hyperlinks>
+    <hyperlink ref="AA2" r:id="rId1"/>
+    <hyperlink ref="AB2" r:id="rId2"/>
+    <hyperlink ref="AC2" r:id="rId3"/>
+    <hyperlink ref="AA3" r:id="rId4"/>
+    <hyperlink ref="AB3" r:id="rId5"/>
+    <hyperlink ref="AC3" r:id="rId6"/>
+    <hyperlink ref="AA4" r:id="rId7"/>
+    <hyperlink ref="AB4" r:id="rId8"/>
+    <hyperlink ref="AC4" r:id="rId9"/>
+    <hyperlink ref="AA5" r:id="rId10"/>
+    <hyperlink ref="AB5" r:id="rId11"/>
+    <hyperlink ref="AC5" r:id="rId12"/>
+    <hyperlink ref="AA6" r:id="rId13"/>
+    <hyperlink ref="AB6" r:id="rId14"/>
+    <hyperlink ref="AC6" r:id="rId15"/>
+    <hyperlink ref="AA7" r:id="rId16"/>
+    <hyperlink ref="AB7" r:id="rId17"/>
+    <hyperlink ref="AC7" r:id="rId18"/>
+    <hyperlink ref="AA8" r:id="rId19"/>
+    <hyperlink ref="AB8" r:id="rId20"/>
+    <hyperlink ref="AC8" r:id="rId21"/>
+    <hyperlink ref="AA9" r:id="rId22"/>
+    <hyperlink ref="AB9" r:id="rId23"/>
+    <hyperlink ref="AC9" r:id="rId24"/>
+    <hyperlink ref="AA10" r:id="rId25"/>
+    <hyperlink ref="AB10" r:id="rId26"/>
+    <hyperlink ref="AC10" r:id="rId27"/>
+    <hyperlink ref="AA11" r:id="rId28"/>
+    <hyperlink ref="AB11" r:id="rId29"/>
+    <hyperlink ref="AC11" r:id="rId30"/>
+    <hyperlink ref="AA12" r:id="rId31"/>
+    <hyperlink ref="AB12" r:id="rId32"/>
+    <hyperlink ref="AC12" r:id="rId33"/>
+    <hyperlink ref="AA13" r:id="rId34"/>
+    <hyperlink ref="AB13" r:id="rId35"/>
+    <hyperlink ref="AC13" r:id="rId36"/>
+    <hyperlink ref="AA14" r:id="rId37"/>
+    <hyperlink ref="AB14" r:id="rId38"/>
+    <hyperlink ref="AC14" r:id="rId39"/>
+    <hyperlink ref="AA15" r:id="rId40"/>
+    <hyperlink ref="AB15" r:id="rId41"/>
+    <hyperlink ref="AC15" r:id="rId42"/>
+    <hyperlink ref="AA16" r:id="rId43"/>
+    <hyperlink ref="AB16" r:id="rId44"/>
+    <hyperlink ref="AC16" r:id="rId45"/>
+    <hyperlink ref="AA17" r:id="rId46"/>
+    <hyperlink ref="AC17" r:id="rId47"/>
+    <hyperlink ref="AA18" r:id="rId48"/>
+    <hyperlink ref="AC18" r:id="rId49"/>
+    <hyperlink ref="AA19" r:id="rId50"/>
+    <hyperlink ref="AC19" r:id="rId51"/>
+    <hyperlink ref="AA20" r:id="rId52"/>
+    <hyperlink ref="AC20" r:id="rId53"/>
+    <hyperlink ref="AA21" r:id="rId54"/>
+    <hyperlink ref="AC21" r:id="rId55"/>
+    <hyperlink ref="AA22" r:id="rId56"/>
+    <hyperlink ref="AC22" r:id="rId57"/>
+    <hyperlink ref="AA23" r:id="rId58"/>
+    <hyperlink ref="AC23" r:id="rId59"/>
+    <hyperlink ref="AA24" r:id="rId60"/>
+    <hyperlink ref="AC24" r:id="rId61"/>
+    <hyperlink ref="AA25" r:id="rId62"/>
+    <hyperlink ref="AC25" r:id="rId63"/>
+    <hyperlink ref="AA26" r:id="rId64"/>
+    <hyperlink ref="AB26" r:id="rId65"/>
+    <hyperlink ref="AC26" r:id="rId66"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AF26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:32" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
@@ -4095,49 +7231,91 @@
         <v>8</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>323</v>
+        <v>478</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>324</v>
+        <v>479</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>325</v>
+        <v>480</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>326</v>
+        <v>481</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>327</v>
+        <v>482</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>328</v>
+        <v>483</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>329</v>
+        <v>484</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>330</v>
+        <v>485</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>331</v>
+        <v>486</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>332</v>
+        <v>487</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>333</v>
+        <v>488</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>334</v>
+        <v>489</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>335</v>
+        <v>490</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>336</v>
+        <v>491</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="AE1" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>505</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -4192,8 +7370,50 @@
       <c r="R2" t="s">
         <v>52</v>
       </c>
+      <c r="S2" t="s">
+        <v>323</v>
+      </c>
+      <c r="T2" t="s">
+        <v>62</v>
+      </c>
+      <c r="U2" t="s">
+        <v>44</v>
+      </c>
+      <c r="V2">
+        <v>50</v>
+      </c>
+      <c r="W2" t="s">
+        <v>192</v>
+      </c>
+      <c r="X2" t="s">
+        <v>326</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA2">
+        <v>28</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>327</v>
+      </c>
+      <c r="AD2">
+        <v>33</v>
+      </c>
+      <c r="AE2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>330</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -4248,8 +7468,50 @@
       <c r="R3" t="s">
         <v>67</v>
       </c>
+      <c r="S3" t="s">
+        <v>334</v>
+      </c>
+      <c r="T3" t="s">
+        <v>61</v>
+      </c>
+      <c r="U3" t="s">
+        <v>44</v>
+      </c>
+      <c r="V3">
+        <v>51</v>
+      </c>
+      <c r="W3" t="s">
+        <v>62</v>
+      </c>
+      <c r="X3" t="s">
+        <v>335</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA3">
+        <v>28</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>336</v>
+      </c>
+      <c r="AD3">
+        <v>31</v>
+      </c>
+      <c r="AE3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>67</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>72</v>
       </c>
@@ -4304,8 +7566,50 @@
       <c r="R4" t="s">
         <v>82</v>
       </c>
+      <c r="S4" t="s">
+        <v>340</v>
+      </c>
+      <c r="T4" t="s">
+        <v>76</v>
+      </c>
+      <c r="U4" t="s">
+        <v>44</v>
+      </c>
+      <c r="V4">
+        <v>12</v>
+      </c>
+      <c r="W4" t="s">
+        <v>62</v>
+      </c>
+      <c r="X4" t="s">
+        <v>341</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA4">
+        <v>7</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>342</v>
+      </c>
+      <c r="AD4">
+        <v>15</v>
+      </c>
+      <c r="AE4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -4360,8 +7664,50 @@
       <c r="R5" t="s">
         <v>93</v>
       </c>
+      <c r="S5" t="s">
+        <v>348</v>
+      </c>
+      <c r="T5" t="s">
+        <v>349</v>
+      </c>
+      <c r="U5" t="s">
+        <v>44</v>
+      </c>
+      <c r="V5">
+        <v>18</v>
+      </c>
+      <c r="W5" t="s">
+        <v>62</v>
+      </c>
+      <c r="X5" t="s">
+        <v>350</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA5">
+        <v>11</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>351</v>
+      </c>
+      <c r="AD5">
+        <v>15</v>
+      </c>
+      <c r="AE5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>93</v>
+      </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>98</v>
       </c>
@@ -4416,8 +7762,50 @@
       <c r="R6" t="s">
         <v>93</v>
       </c>
+      <c r="S6" t="s">
+        <v>355</v>
+      </c>
+      <c r="T6" t="s">
+        <v>100</v>
+      </c>
+      <c r="U6" t="s">
+        <v>44</v>
+      </c>
+      <c r="V6">
+        <v>18</v>
+      </c>
+      <c r="W6" t="s">
+        <v>62</v>
+      </c>
+      <c r="X6" t="s">
+        <v>356</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA6">
+        <v>11</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>357</v>
+      </c>
+      <c r="AD6">
+        <v>14</v>
+      </c>
+      <c r="AE6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>93</v>
+      </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>107</v>
       </c>
@@ -4472,8 +7860,50 @@
       <c r="R7" t="s">
         <v>112</v>
       </c>
+      <c r="S7" t="s">
+        <v>361</v>
+      </c>
+      <c r="T7" t="s">
+        <v>62</v>
+      </c>
+      <c r="U7" t="s">
+        <v>44</v>
+      </c>
+      <c r="V7">
+        <v>24</v>
+      </c>
+      <c r="W7" t="s">
+        <v>62</v>
+      </c>
+      <c r="X7" t="s">
+        <v>362</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA7">
+        <v>12</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>363</v>
+      </c>
+      <c r="AD7">
+        <v>23</v>
+      </c>
+      <c r="AE7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>112</v>
+      </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>117</v>
       </c>
@@ -4528,8 +7958,50 @@
       <c r="R8" t="s">
         <v>124</v>
       </c>
+      <c r="S8" t="s">
+        <v>367</v>
+      </c>
+      <c r="T8" t="s">
+        <v>62</v>
+      </c>
+      <c r="U8" t="s">
+        <v>44</v>
+      </c>
+      <c r="V8">
+        <v>27</v>
+      </c>
+      <c r="W8" t="s">
+        <v>62</v>
+      </c>
+      <c r="X8" t="s">
+        <v>368</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA8">
+        <v>17</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>369</v>
+      </c>
+      <c r="AD8">
+        <v>23</v>
+      </c>
+      <c r="AE8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>371</v>
+      </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>129</v>
       </c>
@@ -4584,8 +8056,50 @@
       <c r="R9" t="s">
         <v>134</v>
       </c>
+      <c r="S9" t="s">
+        <v>375</v>
+      </c>
+      <c r="T9" t="s">
+        <v>61</v>
+      </c>
+      <c r="U9" t="s">
+        <v>44</v>
+      </c>
+      <c r="V9">
+        <v>22</v>
+      </c>
+      <c r="W9" t="s">
+        <v>62</v>
+      </c>
+      <c r="X9" t="s">
+        <v>376</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA9">
+        <v>14</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>377</v>
+      </c>
+      <c r="AD9">
+        <v>22</v>
+      </c>
+      <c r="AE9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>287</v>
+      </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -4640,8 +8154,50 @@
       <c r="R10" t="s">
         <v>146</v>
       </c>
+      <c r="S10" t="s">
+        <v>381</v>
+      </c>
+      <c r="T10" t="s">
+        <v>140</v>
+      </c>
+      <c r="U10" t="s">
+        <v>44</v>
+      </c>
+      <c r="V10">
+        <v>36</v>
+      </c>
+      <c r="W10" t="s">
+        <v>141</v>
+      </c>
+      <c r="X10" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA10">
+        <v>16</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>383</v>
+      </c>
+      <c r="AD10">
+        <v>29</v>
+      </c>
+      <c r="AE10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>146</v>
+      </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>151</v>
       </c>
@@ -4696,8 +8252,50 @@
       <c r="R11" t="s">
         <v>161</v>
       </c>
+      <c r="S11" t="s">
+        <v>387</v>
+      </c>
+      <c r="T11" t="s">
+        <v>62</v>
+      </c>
+      <c r="U11" t="s">
+        <v>44</v>
+      </c>
+      <c r="V11">
+        <v>40</v>
+      </c>
+      <c r="W11" t="s">
+        <v>62</v>
+      </c>
+      <c r="X11" t="s">
+        <v>388</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA11">
+        <v>30</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>389</v>
+      </c>
+      <c r="AD11">
+        <v>39</v>
+      </c>
+      <c r="AE11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>390</v>
+      </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>166</v>
       </c>
@@ -4752,8 +8350,50 @@
       <c r="R12" t="s">
         <v>173</v>
       </c>
+      <c r="S12" t="s">
+        <v>394</v>
+      </c>
+      <c r="T12" t="s">
+        <v>395</v>
+      </c>
+      <c r="U12" t="s">
+        <v>44</v>
+      </c>
+      <c r="V12">
+        <v>26</v>
+      </c>
+      <c r="W12" t="s">
+        <v>62</v>
+      </c>
+      <c r="X12" t="s">
+        <v>396</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA12">
+        <v>22</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>397</v>
+      </c>
+      <c r="AD12">
+        <v>22</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>398</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>399</v>
+      </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>178</v>
       </c>
@@ -4808,8 +8448,50 @@
       <c r="R13" t="s">
         <v>184</v>
       </c>
+      <c r="S13" t="s">
+        <v>403</v>
+      </c>
+      <c r="T13" t="s">
+        <v>404</v>
+      </c>
+      <c r="U13" t="s">
+        <v>44</v>
+      </c>
+      <c r="V13">
+        <v>27</v>
+      </c>
+      <c r="W13" t="s">
+        <v>405</v>
+      </c>
+      <c r="X13" t="s">
+        <v>406</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA13">
+        <v>10</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD13">
+        <v>21</v>
+      </c>
+      <c r="AE13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>409</v>
+      </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>189</v>
       </c>
@@ -4864,8 +8546,50 @@
       <c r="R14" t="s">
         <v>197</v>
       </c>
+      <c r="S14" t="s">
+        <v>413</v>
+      </c>
+      <c r="T14" t="s">
+        <v>191</v>
+      </c>
+      <c r="U14" t="s">
+        <v>44</v>
+      </c>
+      <c r="V14">
+        <v>26</v>
+      </c>
+      <c r="W14" t="s">
+        <v>192</v>
+      </c>
+      <c r="X14" t="s">
+        <v>414</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA14">
+        <v>19</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>415</v>
+      </c>
+      <c r="AD14">
+        <v>17</v>
+      </c>
+      <c r="AE14" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>256</v>
+      </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>202</v>
       </c>
@@ -4920,8 +8644,50 @@
       <c r="R15" t="s">
         <v>207</v>
       </c>
+      <c r="S15" t="s">
+        <v>419</v>
+      </c>
+      <c r="T15" t="s">
+        <v>62</v>
+      </c>
+      <c r="U15" t="s">
+        <v>44</v>
+      </c>
+      <c r="V15">
+        <v>29</v>
+      </c>
+      <c r="W15" t="s">
+        <v>62</v>
+      </c>
+      <c r="X15" t="s">
+        <v>420</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA15">
+        <v>11</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>421</v>
+      </c>
+      <c r="AD15">
+        <v>25</v>
+      </c>
+      <c r="AE15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>207</v>
+      </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>212</v>
       </c>
@@ -4976,8 +8742,50 @@
       <c r="R16" t="s">
         <v>217</v>
       </c>
+      <c r="S16" t="s">
+        <v>425</v>
+      </c>
+      <c r="T16" t="s">
+        <v>62</v>
+      </c>
+      <c r="U16" t="s">
+        <v>44</v>
+      </c>
+      <c r="V16">
+        <v>34</v>
+      </c>
+      <c r="W16" t="s">
+        <v>62</v>
+      </c>
+      <c r="X16" t="s">
+        <v>426</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA16">
+        <v>25</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD16">
+        <v>24</v>
+      </c>
+      <c r="AE16" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>217</v>
+      </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>222</v>
       </c>
@@ -5032,8 +8840,50 @@
       <c r="R17" t="s">
         <v>44</v>
       </c>
+      <c r="S17" t="s">
+        <v>431</v>
+      </c>
+      <c r="T17" t="s">
+        <v>432</v>
+      </c>
+      <c r="U17" t="s">
+        <v>44</v>
+      </c>
+      <c r="V17">
+        <v>36</v>
+      </c>
+      <c r="W17" t="s">
+        <v>62</v>
+      </c>
+      <c r="X17" t="s">
+        <v>433</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD17">
+        <v>20</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>232</v>
       </c>
@@ -5088,8 +8938,50 @@
       <c r="R18" t="s">
         <v>44</v>
       </c>
+      <c r="S18" t="s">
+        <v>436</v>
+      </c>
+      <c r="T18" t="s">
+        <v>234</v>
+      </c>
+      <c r="U18" t="s">
+        <v>44</v>
+      </c>
+      <c r="V18">
+        <v>16</v>
+      </c>
+      <c r="W18" t="s">
+        <v>62</v>
+      </c>
+      <c r="X18" t="s">
+        <v>437</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD18">
+        <v>8</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>239</v>
       </c>
@@ -5144,8 +9036,50 @@
       <c r="R19" t="s">
         <v>44</v>
       </c>
+      <c r="S19" t="s">
+        <v>440</v>
+      </c>
+      <c r="T19" t="s">
+        <v>441</v>
+      </c>
+      <c r="U19" t="s">
+        <v>44</v>
+      </c>
+      <c r="V19">
+        <v>47</v>
+      </c>
+      <c r="W19" t="s">
+        <v>45</v>
+      </c>
+      <c r="X19" t="s">
+        <v>442</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD19">
+        <v>18</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>246</v>
       </c>
@@ -5200,8 +9134,50 @@
       <c r="R20" t="s">
         <v>256</v>
       </c>
+      <c r="S20" t="s">
+        <v>445</v>
+      </c>
+      <c r="T20" t="s">
+        <v>251</v>
+      </c>
+      <c r="U20" t="s">
+        <v>44</v>
+      </c>
+      <c r="V20">
+        <v>26</v>
+      </c>
+      <c r="W20" t="s">
+        <v>62</v>
+      </c>
+      <c r="X20" t="s">
+        <v>446</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD20">
+        <v>21</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>261</v>
       </c>
@@ -5256,8 +9232,50 @@
       <c r="R21" t="s">
         <v>173</v>
       </c>
+      <c r="S21" t="s">
+        <v>449</v>
+      </c>
+      <c r="T21" t="s">
+        <v>293</v>
+      </c>
+      <c r="U21" t="s">
+        <v>44</v>
+      </c>
+      <c r="V21">
+        <v>12</v>
+      </c>
+      <c r="W21" t="s">
+        <v>62</v>
+      </c>
+      <c r="X21" t="s">
+        <v>450</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD21">
+        <v>10</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>271</v>
       </c>
@@ -5312,8 +9330,50 @@
       <c r="R22" t="s">
         <v>276</v>
       </c>
+      <c r="S22" t="s">
+        <v>453</v>
+      </c>
+      <c r="T22" t="s">
+        <v>251</v>
+      </c>
+      <c r="U22" t="s">
+        <v>44</v>
+      </c>
+      <c r="V22">
+        <v>14</v>
+      </c>
+      <c r="W22" t="s">
+        <v>62</v>
+      </c>
+      <c r="X22" t="s">
+        <v>454</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD22">
+        <v>11</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>281</v>
       </c>
@@ -5368,8 +9428,50 @@
       <c r="R23" t="s">
         <v>287</v>
       </c>
+      <c r="S23" t="s">
+        <v>457</v>
+      </c>
+      <c r="T23" t="s">
+        <v>251</v>
+      </c>
+      <c r="U23" t="s">
+        <v>44</v>
+      </c>
+      <c r="V23">
+        <v>22</v>
+      </c>
+      <c r="W23" t="s">
+        <v>62</v>
+      </c>
+      <c r="X23" t="s">
+        <v>458</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD23">
+        <v>18</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>292</v>
       </c>
@@ -5424,8 +9526,50 @@
       <c r="R24" t="s">
         <v>44</v>
       </c>
+      <c r="S24" t="s">
+        <v>461</v>
+      </c>
+      <c r="T24" t="s">
+        <v>293</v>
+      </c>
+      <c r="U24" t="s">
+        <v>44</v>
+      </c>
+      <c r="V24">
+        <v>8</v>
+      </c>
+      <c r="W24" t="s">
+        <v>62</v>
+      </c>
+      <c r="X24" t="s">
+        <v>462</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD24">
+        <v>7</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>298</v>
       </c>
@@ -5480,8 +9624,50 @@
       <c r="R25" t="s">
         <v>303</v>
       </c>
+      <c r="S25" t="s">
+        <v>465</v>
+      </c>
+      <c r="T25" t="s">
+        <v>62</v>
+      </c>
+      <c r="U25" t="s">
+        <v>44</v>
+      </c>
+      <c r="V25">
+        <v>4</v>
+      </c>
+      <c r="W25" t="s">
+        <v>62</v>
+      </c>
+      <c r="X25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD25">
+        <v>3</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>308</v>
       </c>
@@ -5536,9 +9722,51 @@
       <c r="R26" t="s">
         <v>319</v>
       </c>
+      <c r="S26" t="s">
+        <v>469</v>
+      </c>
+      <c r="T26" t="s">
+        <v>470</v>
+      </c>
+      <c r="U26" t="s">
+        <v>44</v>
+      </c>
+      <c r="V26">
+        <v>25</v>
+      </c>
+      <c r="W26" t="s">
+        <v>45</v>
+      </c>
+      <c r="X26" t="s">
+        <v>471</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>315</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA26">
+        <v>7</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>472</v>
+      </c>
+      <c r="AD26">
+        <v>13</v>
+      </c>
+      <c r="AE26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>474</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
+  <autoFilter ref="A1:AF1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>